<commit_message>
Added rational for mapping co-pso dcn subject, need to add ut1-2 marks
</commit_message>
<xml_diff>
--- a/Attainment Calculation/Sheet from BRC for Attainment Calculation/CR 3 _DATA COMMUNICATION AND COMPUTER NETWORK(314318).xlsx
+++ b/Attainment Calculation/Sheet from BRC for Attainment Calculation/CR 3 _DATA COMMUNICATION AND COMPUTER NETWORK(314318).xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="645" windowWidth="10065" windowHeight="9660" activeTab="3"/>
+    <workbookView xWindow="390" yWindow="645" windowWidth="10065" windowHeight="9660" firstSheet="3" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="PO Set Target attain level" sheetId="1" r:id="rId1"/>
@@ -3298,10 +3298,58 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3315,26 +3363,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3351,20 +3379,10 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3373,6 +3391,9 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3402,15 +3423,19 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3430,33 +3455,54 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="24" fillId="3" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3469,22 +3515,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="24" fillId="3" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3496,17 +3531,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="78" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="79" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3533,6 +3557,14 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="78" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="79" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3636,38 +3668,6 @@
     <xf numFmtId="2" fontId="3" fillId="3" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4340,40 +4340,40 @@
       <c r="C3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="213" t="s">
+      <c r="D3" s="223" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="208"/>
+      <c r="E3" s="209"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B4" s="6"/>
       <c r="C4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="213">
+      <c r="D4" s="223">
         <v>314318</v>
       </c>
-      <c r="E4" s="208"/>
+      <c r="E4" s="209"/>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B5" s="4"/>
       <c r="C5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="214" t="s">
+      <c r="D5" s="224" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="207"/>
+      <c r="E5" s="208"/>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B6" s="4"/>
       <c r="C6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="213" t="s">
+      <c r="D6" s="223" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="208"/>
+      <c r="E6" s="209"/>
     </row>
     <row r="7" spans="2:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B7" s="7" t="s">
@@ -4388,50 +4388,50 @@
       <c r="C8" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="188" t="s">
+      <c r="D8" s="225" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="189"/>
+      <c r="E8" s="226"/>
     </row>
     <row r="9" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="6"/>
       <c r="C9" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="188" t="s">
+      <c r="D9" s="225" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="189"/>
+      <c r="E9" s="226"/>
     </row>
     <row r="10" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="6"/>
       <c r="C10" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="188" t="s">
+      <c r="D10" s="225" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="189"/>
+      <c r="E10" s="226"/>
     </row>
     <row r="11" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="6"/>
       <c r="C11" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="188" t="s">
+      <c r="D11" s="225" t="s">
         <v>16</v>
       </c>
-      <c r="E11" s="189"/>
+      <c r="E11" s="226"/>
     </row>
     <row r="12" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="6"/>
       <c r="C12" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="188" t="s">
+      <c r="D12" s="225" t="s">
         <v>18</v>
       </c>
-      <c r="E12" s="189"/>
+      <c r="E12" s="226"/>
     </row>
     <row r="14" spans="2:13" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
@@ -4466,31 +4466,31 @@
       <c r="M15" s="11"/>
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B16" s="190" t="s">
+      <c r="B16" s="210" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="193" t="s">
+      <c r="C16" s="213" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="194"/>
-      <c r="E16" s="199" t="s">
+      <c r="D16" s="214"/>
+      <c r="E16" s="200" t="s">
         <v>23</v>
       </c>
-      <c r="F16" s="200"/>
-      <c r="G16" s="200"/>
-      <c r="H16" s="200"/>
-      <c r="I16" s="200"/>
-      <c r="J16" s="200"/>
+      <c r="F16" s="203"/>
+      <c r="G16" s="203"/>
+      <c r="H16" s="203"/>
+      <c r="I16" s="203"/>
+      <c r="J16" s="203"/>
       <c r="K16" s="201"/>
-      <c r="L16" s="199" t="s">
+      <c r="L16" s="200" t="s">
         <v>24</v>
       </c>
       <c r="M16" s="201"/>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B17" s="191"/>
-      <c r="C17" s="195"/>
-      <c r="D17" s="196"/>
+      <c r="B17" s="211"/>
+      <c r="C17" s="215"/>
+      <c r="D17" s="216"/>
       <c r="E17" s="13" t="s">
         <v>25</v>
       </c>
@@ -4520,9 +4520,9 @@
       </c>
     </row>
     <row r="18" spans="1:25" ht="122.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="192"/>
-      <c r="C18" s="197"/>
-      <c r="D18" s="198"/>
+      <c r="B18" s="212"/>
+      <c r="C18" s="217"/>
+      <c r="D18" s="218"/>
       <c r="E18" s="14" t="s">
         <v>34</v>
       </c>
@@ -4755,7 +4755,7 @@
       <c r="B24" s="202" t="s">
         <v>44</v>
       </c>
-      <c r="C24" s="200"/>
+      <c r="C24" s="203"/>
       <c r="D24" s="201"/>
       <c r="E24" s="16">
         <f t="shared" ref="E24:M24" si="5">IFERROR(AVERAGE(E19:E23),2)</f>
@@ -4795,10 +4795,10 @@
       </c>
     </row>
     <row r="25" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="203" t="s">
+      <c r="B25" s="204" t="s">
         <v>45</v>
       </c>
-      <c r="C25" s="200"/>
+      <c r="C25" s="203"/>
       <c r="D25" s="201"/>
       <c r="E25" s="22">
         <f t="shared" ref="E25:M25" si="6">E24</f>
@@ -4843,32 +4843,32 @@
       <c r="D28" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="I28" s="204" t="s">
+      <c r="I28" s="205" t="s">
         <v>47</v>
       </c>
-      <c r="J28" s="205"/>
-      <c r="K28" s="205"/>
-      <c r="L28" s="205"/>
-      <c r="M28" s="205"/>
+      <c r="J28" s="206"/>
+      <c r="K28" s="206"/>
+      <c r="L28" s="206"/>
+      <c r="M28" s="206"/>
     </row>
     <row r="29" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="25"/>
       <c r="B29" s="25"/>
-      <c r="C29" s="206" t="s">
+      <c r="C29" s="207" t="s">
         <v>48</v>
       </c>
-      <c r="D29" s="207"/>
-      <c r="E29" s="208"/>
+      <c r="D29" s="208"/>
+      <c r="E29" s="209"/>
       <c r="F29" s="25"/>
       <c r="G29" s="25"/>
       <c r="H29" s="25"/>
-      <c r="I29" s="206" t="s">
+      <c r="I29" s="207" t="s">
         <v>48</v>
       </c>
-      <c r="J29" s="207"/>
-      <c r="K29" s="207"/>
-      <c r="L29" s="207"/>
-      <c r="M29" s="208"/>
+      <c r="J29" s="208"/>
+      <c r="K29" s="208"/>
+      <c r="L29" s="208"/>
+      <c r="M29" s="209"/>
       <c r="N29" s="25"/>
       <c r="O29" s="25"/>
       <c r="P29" s="25"/>
@@ -4886,22 +4886,22 @@
     <row r="31" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="32" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="33" spans="2:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="209" t="s">
+      <c r="B33" s="219" t="s">
         <v>49</v>
       </c>
       <c r="C33" s="20"/>
-      <c r="D33" s="211" t="s">
+      <c r="D33" s="221" t="s">
         <v>50</v>
       </c>
-      <c r="E33" s="205"/>
+      <c r="E33" s="206"/>
     </row>
     <row r="34" spans="2:5" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="210"/>
+      <c r="B34" s="220"/>
       <c r="C34" s="22"/>
-      <c r="D34" s="212" t="s">
+      <c r="D34" s="222" t="s">
         <v>51</v>
       </c>
-      <c r="E34" s="205"/>
+      <c r="E34" s="206"/>
     </row>
     <row r="35" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="36" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -5881,14 +5881,14 @@
     <mergeCell ref="D8:E8"/>
     <mergeCell ref="D9:E9"/>
     <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
     <mergeCell ref="L16:M16"/>
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="B25:D25"/>
     <mergeCell ref="I28:M28"/>
     <mergeCell ref="C29:E29"/>
     <mergeCell ref="I29:M29"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
     <mergeCell ref="B16:B18"/>
     <mergeCell ref="C16:D18"/>
     <mergeCell ref="E16:K16"/>
@@ -5909,139 +5909,139 @@
     <col min="4" max="4" width="47.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="B4" s="326" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B4" s="188" t="s">
         <v>256</v>
       </c>
-      <c r="C4" s="326" t="s">
+      <c r="C4" s="188" t="s">
         <v>257</v>
       </c>
-      <c r="D4" s="326" t="s">
+      <c r="D4" s="188" t="s">
         <v>258</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="326" t="s">
+      <c r="B5" s="188" t="s">
         <v>259</v>
       </c>
-      <c r="C5" s="327">
+      <c r="C5" s="189">
         <v>2</v>
       </c>
-      <c r="D5" s="327">
+      <c r="D5" s="189">
         <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="326" t="s">
+      <c r="B6" s="188" t="s">
         <v>260</v>
       </c>
-      <c r="C6" s="327">
+      <c r="C6" s="189">
         <v>1</v>
       </c>
-      <c r="D6" s="327">
+      <c r="D6" s="189">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="326" t="s">
+      <c r="B7" s="188" t="s">
         <v>261</v>
       </c>
-      <c r="C7" s="327">
+      <c r="C7" s="189">
         <v>1</v>
       </c>
-      <c r="D7" s="327">
+      <c r="D7" s="189">
         <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="326" t="s">
+      <c r="B8" s="188" t="s">
         <v>262</v>
       </c>
-      <c r="C8" s="327">
+      <c r="C8" s="189">
         <v>2</v>
       </c>
-      <c r="D8" s="327">
+      <c r="D8" s="189">
         <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="326" t="s">
+      <c r="B9" s="188" t="s">
         <v>263</v>
       </c>
-      <c r="C9" s="327">
+      <c r="C9" s="189">
         <v>2</v>
       </c>
-      <c r="D9" s="327">
+      <c r="D9" s="189">
         <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="18" x14ac:dyDescent="0.25">
-      <c r="A12" s="329" t="s">
+      <c r="A12" s="191" t="s">
         <v>264</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="330"/>
+      <c r="A13" s="192"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="334" t="s">
+      <c r="A14" s="196" t="s">
         <v>265</v>
       </c>
-      <c r="B14" s="335"/>
+      <c r="B14" s="197"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="331"/>
+      <c r="A15" s="193"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="332" t="s">
+      <c r="A16" s="194" t="s">
         <v>269</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="331"/>
+      <c r="A17" s="193"/>
       <c r="B17" t="s">
         <v>270</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="331"/>
+      <c r="A18" s="193"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="332" t="s">
+      <c r="A19" s="194" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="330"/>
+      <c r="A20" s="192"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="334" t="s">
+      <c r="A21" s="196" t="s">
         <v>267</v>
       </c>
-      <c r="B21" s="335"/>
+      <c r="B21" s="197"/>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="331"/>
+      <c r="A22" s="193"/>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="333" t="s">
+      <c r="A23" s="195" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="328"/>
+      <c r="A24" s="190"/>
       <c r="B24" t="s">
         <v>273</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="328"/>
+      <c r="A25" s="190"/>
       <c r="B25" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="333" t="s">
+      <c r="A26" s="195" t="s">
         <v>268</v>
       </c>
     </row>
@@ -6074,38 +6074,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="21.75" x14ac:dyDescent="0.35">
-      <c r="A1" s="240" t="s">
+      <c r="A1" s="251" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="205"/>
-      <c r="C1" s="205"/>
-      <c r="D1" s="205"/>
-      <c r="E1" s="205"/>
-      <c r="F1" s="205"/>
-      <c r="G1" s="205"/>
-      <c r="H1" s="205"/>
-      <c r="I1" s="205"/>
-      <c r="J1" s="205"/>
-      <c r="K1" s="205"/>
+      <c r="B1" s="206"/>
+      <c r="C1" s="206"/>
+      <c r="D1" s="206"/>
+      <c r="E1" s="206"/>
+      <c r="F1" s="206"/>
+      <c r="G1" s="206"/>
+      <c r="H1" s="206"/>
+      <c r="I1" s="206"/>
+      <c r="J1" s="206"/>
+      <c r="K1" s="206"/>
       <c r="L1" s="6"/>
       <c r="M1" s="6"/>
       <c r="N1" s="6"/>
       <c r="O1" s="6"/>
     </row>
     <row r="2" spans="1:15" ht="21.75" x14ac:dyDescent="0.35">
-      <c r="A2" s="240" t="s">
+      <c r="A2" s="251" t="s">
         <v>53</v>
       </c>
-      <c r="B2" s="205"/>
-      <c r="C2" s="205"/>
-      <c r="D2" s="205"/>
-      <c r="E2" s="205"/>
-      <c r="F2" s="205"/>
-      <c r="G2" s="205"/>
-      <c r="H2" s="205"/>
-      <c r="I2" s="205"/>
-      <c r="J2" s="205"/>
-      <c r="K2" s="205"/>
+      <c r="B2" s="206"/>
+      <c r="C2" s="206"/>
+      <c r="D2" s="206"/>
+      <c r="E2" s="206"/>
+      <c r="F2" s="206"/>
+      <c r="G2" s="206"/>
+      <c r="H2" s="206"/>
+      <c r="I2" s="206"/>
+      <c r="J2" s="206"/>
+      <c r="K2" s="206"/>
       <c r="L2" s="6"/>
       <c r="M2" s="6"/>
       <c r="N2" s="6"/>
@@ -6116,11 +6116,11 @@
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="241" t="str">
+      <c r="C3" s="252" t="str">
         <f>'PO Set Target attain level'!D3</f>
         <v>Data Communication and Computer Network (DCN)</v>
       </c>
-      <c r="D3" s="189"/>
+      <c r="D3" s="226"/>
       <c r="E3" s="6"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
@@ -6138,11 +6138,11 @@
       <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="241">
+      <c r="C4" s="252">
         <f>'PO Set Target attain level'!D4</f>
         <v>314318</v>
       </c>
-      <c r="D4" s="189"/>
+      <c r="D4" s="226"/>
       <c r="E4" s="6"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
@@ -6160,11 +6160,11 @@
       <c r="B5" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C5" s="241" t="str">
+      <c r="C5" s="252" t="str">
         <f>'PO Set Target attain level'!D5</f>
         <v>4th Sem Co4K K-Scheme</v>
       </c>
-      <c r="D5" s="189"/>
+      <c r="D5" s="226"/>
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
@@ -6182,11 +6182,11 @@
       <c r="B6" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="241" t="str">
+      <c r="C6" s="252" t="str">
         <f>'PO Set Target attain level'!D6</f>
         <v>2024-25</v>
       </c>
-      <c r="D6" s="189"/>
+      <c r="D6" s="226"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -6217,31 +6217,31 @@
       <c r="O7" s="6"/>
     </row>
     <row r="8" spans="1:15" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="242" t="s">
+      <c r="A8" s="253" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="219" t="s">
+      <c r="B8" s="261" t="s">
         <v>56</v>
       </c>
-      <c r="C8" s="220" t="s">
+      <c r="C8" s="262" t="s">
         <v>57</v>
       </c>
-      <c r="D8" s="236" t="s">
+      <c r="D8" s="263" t="s">
         <v>58</v>
       </c>
-      <c r="E8" s="237" t="s">
+      <c r="E8" s="264" t="s">
         <v>59</v>
       </c>
-      <c r="F8" s="215" t="s">
+      <c r="F8" s="259" t="s">
         <v>60</v>
       </c>
-      <c r="G8" s="218" t="s">
+      <c r="G8" s="260" t="s">
         <v>61</v>
       </c>
-      <c r="H8" s="238" t="s">
+      <c r="H8" s="247" t="s">
         <v>62</v>
       </c>
-      <c r="I8" s="239" t="s">
+      <c r="I8" s="250" t="s">
         <v>63</v>
       </c>
       <c r="J8" s="26" t="s">
@@ -6256,62 +6256,62 @@
       <c r="O8" s="6"/>
     </row>
     <row r="9" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="216"/>
-      <c r="B9" s="216"/>
-      <c r="C9" s="216"/>
-      <c r="D9" s="216"/>
-      <c r="E9" s="216"/>
-      <c r="F9" s="216"/>
-      <c r="G9" s="216"/>
-      <c r="H9" s="216"/>
-      <c r="I9" s="216"/>
-      <c r="J9" s="243" t="s">
+      <c r="A9" s="248"/>
+      <c r="B9" s="248"/>
+      <c r="C9" s="248"/>
+      <c r="D9" s="248"/>
+      <c r="E9" s="248"/>
+      <c r="F9" s="248"/>
+      <c r="G9" s="248"/>
+      <c r="H9" s="248"/>
+      <c r="I9" s="248"/>
+      <c r="J9" s="254" t="s">
         <v>66</v>
       </c>
-      <c r="K9" s="244"/>
+      <c r="K9" s="255"/>
       <c r="L9" s="6"/>
       <c r="M9" s="6"/>
       <c r="N9" s="6"/>
       <c r="O9" s="6"/>
     </row>
     <row r="10" spans="1:15" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="216"/>
-      <c r="B10" s="216"/>
-      <c r="C10" s="216"/>
-      <c r="D10" s="216"/>
-      <c r="E10" s="216"/>
-      <c r="F10" s="216"/>
-      <c r="G10" s="216"/>
-      <c r="H10" s="216"/>
-      <c r="I10" s="216"/>
-      <c r="J10" s="245"/>
-      <c r="K10" s="210"/>
+      <c r="A10" s="248"/>
+      <c r="B10" s="248"/>
+      <c r="C10" s="248"/>
+      <c r="D10" s="248"/>
+      <c r="E10" s="248"/>
+      <c r="F10" s="248"/>
+      <c r="G10" s="248"/>
+      <c r="H10" s="248"/>
+      <c r="I10" s="248"/>
+      <c r="J10" s="256"/>
+      <c r="K10" s="220"/>
       <c r="L10" s="6"/>
       <c r="M10" s="6"/>
       <c r="N10" s="6"/>
       <c r="O10" s="6"/>
     </row>
     <row r="11" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="216"/>
-      <c r="B11" s="216"/>
-      <c r="C11" s="216"/>
-      <c r="D11" s="217"/>
-      <c r="E11" s="217"/>
-      <c r="F11" s="217"/>
-      <c r="G11" s="217"/>
-      <c r="H11" s="217"/>
-      <c r="I11" s="217"/>
-      <c r="J11" s="246"/>
-      <c r="K11" s="247"/>
+      <c r="A11" s="248"/>
+      <c r="B11" s="248"/>
+      <c r="C11" s="248"/>
+      <c r="D11" s="249"/>
+      <c r="E11" s="249"/>
+      <c r="F11" s="249"/>
+      <c r="G11" s="249"/>
+      <c r="H11" s="249"/>
+      <c r="I11" s="249"/>
+      <c r="J11" s="257"/>
+      <c r="K11" s="258"/>
       <c r="L11" s="6"/>
       <c r="M11" s="6"/>
       <c r="N11" s="6"/>
       <c r="O11" s="6"/>
     </row>
     <row r="12" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="217"/>
-      <c r="B12" s="217"/>
-      <c r="C12" s="217"/>
+      <c r="A12" s="249"/>
+      <c r="B12" s="249"/>
+      <c r="C12" s="249"/>
       <c r="D12" s="27">
         <v>8</v>
       </c>
@@ -8696,93 +8696,93 @@
       <c r="O95" s="6"/>
     </row>
     <row r="96" spans="1:15" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="221" t="s">
+      <c r="A96" s="227" t="s">
         <v>137</v>
       </c>
-      <c r="B96" s="205"/>
+      <c r="B96" s="206"/>
       <c r="C96" s="41">
         <v>0.4</v>
       </c>
-      <c r="D96" s="222">
+      <c r="D96" s="228">
         <f t="shared" ref="D96:I96" si="5">$C$96*D12</f>
         <v>3.2</v>
       </c>
-      <c r="E96" s="222">
+      <c r="E96" s="228">
         <f t="shared" si="5"/>
         <v>4.8000000000000007</v>
       </c>
-      <c r="F96" s="222">
+      <c r="F96" s="228">
         <f t="shared" si="5"/>
         <v>3.2</v>
       </c>
-      <c r="G96" s="222">
+      <c r="G96" s="228">
         <f t="shared" si="5"/>
         <v>3.2</v>
       </c>
-      <c r="H96" s="222">
+      <c r="H96" s="228">
         <f t="shared" si="5"/>
         <v>4.8000000000000007</v>
       </c>
-      <c r="I96" s="222">
+      <c r="I96" s="228">
         <f t="shared" si="5"/>
         <v>3.2</v>
       </c>
-      <c r="J96" s="248"/>
-      <c r="K96" s="248"/>
+      <c r="J96" s="265"/>
+      <c r="K96" s="265"/>
       <c r="L96" s="6"/>
       <c r="M96" s="6"/>
       <c r="N96" s="6"/>
       <c r="O96" s="6"/>
     </row>
     <row r="97" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="223" t="s">
+      <c r="A97" s="229" t="s">
         <v>138</v>
       </c>
-      <c r="B97" s="205"/>
-      <c r="C97" s="196"/>
-      <c r="D97" s="192"/>
-      <c r="E97" s="192"/>
-      <c r="F97" s="192"/>
-      <c r="G97" s="192"/>
-      <c r="H97" s="192"/>
-      <c r="I97" s="192"/>
-      <c r="J97" s="192"/>
-      <c r="K97" s="192"/>
+      <c r="B97" s="206"/>
+      <c r="C97" s="216"/>
+      <c r="D97" s="212"/>
+      <c r="E97" s="212"/>
+      <c r="F97" s="212"/>
+      <c r="G97" s="212"/>
+      <c r="H97" s="212"/>
+      <c r="I97" s="212"/>
+      <c r="J97" s="212"/>
+      <c r="K97" s="212"/>
       <c r="L97" s="6"/>
       <c r="M97" s="6"/>
       <c r="N97" s="6"/>
       <c r="O97" s="6"/>
     </row>
     <row r="98" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A98" s="205"/>
-      <c r="B98" s="205"/>
-      <c r="C98" s="196"/>
-      <c r="D98" s="250">
+      <c r="A98" s="206"/>
+      <c r="B98" s="206"/>
+      <c r="C98" s="216"/>
+      <c r="D98" s="230">
         <f t="shared" ref="D98:I98" si="6">COUNTIF(D13:D95,"&gt;=" &amp;D96)</f>
         <v>0</v>
       </c>
-      <c r="E98" s="250">
+      <c r="E98" s="230">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="F98" s="250">
+      <c r="F98" s="230">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G98" s="250">
+      <c r="G98" s="230">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="H98" s="250">
+      <c r="H98" s="230">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="I98" s="250">
+      <c r="I98" s="230">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="J98" s="249"/>
-      <c r="K98" s="249"/>
+      <c r="J98" s="266"/>
+      <c r="K98" s="266"/>
       <c r="L98" s="6"/>
       <c r="M98" s="6"/>
       <c r="N98" s="6"/>
@@ -8792,14 +8792,14 @@
       <c r="A99" s="6"/>
       <c r="B99" s="6"/>
       <c r="C99" s="6"/>
-      <c r="D99" s="192"/>
-      <c r="E99" s="192"/>
-      <c r="F99" s="192"/>
-      <c r="G99" s="192"/>
-      <c r="H99" s="192"/>
-      <c r="I99" s="192"/>
-      <c r="J99" s="192"/>
-      <c r="K99" s="192"/>
+      <c r="D99" s="212"/>
+      <c r="E99" s="212"/>
+      <c r="F99" s="212"/>
+      <c r="G99" s="212"/>
+      <c r="H99" s="212"/>
+      <c r="I99" s="212"/>
+      <c r="J99" s="212"/>
+      <c r="K99" s="212"/>
       <c r="L99" s="6"/>
       <c r="M99" s="6"/>
       <c r="N99" s="6"/>
@@ -8858,18 +8858,18 @@
     </row>
     <row r="103" spans="1:15" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="6"/>
-      <c r="B103" s="229" t="s">
+      <c r="B103" s="236" t="s">
         <v>139</v>
       </c>
-      <c r="C103" s="200"/>
-      <c r="D103" s="200"/>
+      <c r="C103" s="203"/>
+      <c r="D103" s="203"/>
       <c r="E103" s="201"/>
-      <c r="F103" s="230" t="s">
+      <c r="F103" s="237" t="s">
         <v>140</v>
       </c>
       <c r="G103" s="201"/>
       <c r="H103" s="42"/>
-      <c r="I103" s="231" t="s">
+      <c r="I103" s="238" t="s">
         <v>141</v>
       </c>
       <c r="J103" s="201"/>
@@ -8881,28 +8881,28 @@
     </row>
     <row r="104" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="6"/>
-      <c r="B104" s="232" t="s">
+      <c r="B104" s="239" t="s">
         <v>142</v>
       </c>
-      <c r="C104" s="224" t="s">
+      <c r="C104" s="231" t="s">
         <v>143</v>
       </c>
-      <c r="D104" s="225"/>
+      <c r="D104" s="232"/>
       <c r="E104" s="43">
         <v>50</v>
       </c>
-      <c r="F104" s="235">
+      <c r="F104" s="242">
         <v>70</v>
       </c>
-      <c r="G104" s="194"/>
+      <c r="G104" s="214"/>
       <c r="H104" s="44">
         <f>E104*F104/100</f>
         <v>35</v>
       </c>
-      <c r="I104" s="251">
+      <c r="I104" s="243">
         <v>1</v>
       </c>
-      <c r="J104" s="252"/>
+      <c r="J104" s="244"/>
       <c r="K104" s="6"/>
       <c r="L104" s="6"/>
       <c r="M104" s="6"/>
@@ -8911,24 +8911,24 @@
     </row>
     <row r="105" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="6"/>
-      <c r="B105" s="233"/>
-      <c r="C105" s="224" t="s">
+      <c r="B105" s="240"/>
+      <c r="C105" s="231" t="s">
         <v>143</v>
       </c>
-      <c r="D105" s="225"/>
+      <c r="D105" s="232"/>
       <c r="E105" s="43">
         <v>60</v>
       </c>
-      <c r="F105" s="195"/>
-      <c r="G105" s="196"/>
+      <c r="F105" s="215"/>
+      <c r="G105" s="216"/>
       <c r="H105" s="45">
         <f>E105*F104/100</f>
         <v>42</v>
       </c>
-      <c r="I105" s="253">
+      <c r="I105" s="245">
         <v>2</v>
       </c>
-      <c r="J105" s="254"/>
+      <c r="J105" s="246"/>
       <c r="K105" s="6"/>
       <c r="L105" s="6"/>
       <c r="M105" s="6"/>
@@ -8937,24 +8937,24 @@
     </row>
     <row r="106" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="6"/>
-      <c r="B106" s="234"/>
-      <c r="C106" s="224" t="s">
+      <c r="B106" s="241"/>
+      <c r="C106" s="231" t="s">
         <v>143</v>
       </c>
-      <c r="D106" s="225"/>
+      <c r="D106" s="232"/>
       <c r="E106" s="46">
         <v>70</v>
       </c>
-      <c r="F106" s="197"/>
-      <c r="G106" s="198"/>
+      <c r="F106" s="217"/>
+      <c r="G106" s="218"/>
       <c r="H106" s="47">
         <f>E106*F104/100</f>
         <v>49</v>
       </c>
-      <c r="I106" s="226">
+      <c r="I106" s="233">
         <v>3</v>
       </c>
-      <c r="J106" s="227"/>
+      <c r="J106" s="234"/>
       <c r="K106" s="6"/>
       <c r="L106" s="6"/>
       <c r="M106" s="6"/>
@@ -8969,9 +8969,9 @@
       <c r="E107" s="48"/>
       <c r="F107" s="48"/>
       <c r="G107" s="48"/>
-      <c r="H107" s="228"/>
-      <c r="I107" s="207"/>
-      <c r="J107" s="208"/>
+      <c r="H107" s="235"/>
+      <c r="I107" s="208"/>
+      <c r="J107" s="209"/>
       <c r="K107" s="6"/>
       <c r="L107" s="6"/>
       <c r="M107" s="6"/>
@@ -8986,9 +8986,9 @@
       <c r="E108" s="48"/>
       <c r="F108" s="48"/>
       <c r="G108" s="48"/>
-      <c r="H108" s="228"/>
-      <c r="I108" s="207"/>
-      <c r="J108" s="208"/>
+      <c r="H108" s="235"/>
+      <c r="I108" s="208"/>
+      <c r="J108" s="209"/>
       <c r="K108" s="6"/>
       <c r="L108" s="6"/>
       <c r="M108" s="6"/>
@@ -13351,6 +13351,12 @@
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A8:A12"/>
     <mergeCell ref="J9:K11"/>
+    <mergeCell ref="F8:F11"/>
+    <mergeCell ref="G8:G11"/>
+    <mergeCell ref="B8:B12"/>
+    <mergeCell ref="C8:C12"/>
+    <mergeCell ref="D8:D11"/>
+    <mergeCell ref="E8:E11"/>
     <mergeCell ref="C106:D106"/>
     <mergeCell ref="I106:J106"/>
     <mergeCell ref="H107:J107"/>
@@ -13364,17 +13370,11 @@
     <mergeCell ref="C105:D105"/>
     <mergeCell ref="I104:J104"/>
     <mergeCell ref="I105:J105"/>
-    <mergeCell ref="F8:F11"/>
-    <mergeCell ref="G8:G11"/>
-    <mergeCell ref="B8:B12"/>
-    <mergeCell ref="C8:C12"/>
     <mergeCell ref="A96:B96"/>
     <mergeCell ref="E96:E97"/>
     <mergeCell ref="F96:F97"/>
     <mergeCell ref="G96:G97"/>
     <mergeCell ref="A97:C98"/>
-    <mergeCell ref="D8:D11"/>
-    <mergeCell ref="E8:E11"/>
     <mergeCell ref="D96:D97"/>
     <mergeCell ref="D98:D99"/>
     <mergeCell ref="E98:E99"/>
@@ -13405,13 +13405,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:22" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="B1" s="255" t="s">
+      <c r="B1" s="267" t="s">
         <v>149</v>
       </c>
-      <c r="C1" s="205"/>
-      <c r="D1" s="205"/>
-      <c r="E1" s="205"/>
-      <c r="F1" s="205"/>
+      <c r="C1" s="206"/>
+      <c r="D1" s="206"/>
+      <c r="E1" s="206"/>
+      <c r="F1" s="206"/>
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
@@ -13480,11 +13480,11 @@
       <c r="C4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="256" t="str">
+      <c r="D4" s="268" t="str">
         <f>'CO_Attainment for Unit Tests'!C3</f>
         <v>Data Communication and Computer Network (DCN)</v>
       </c>
-      <c r="E4" s="208"/>
+      <c r="E4" s="209"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
@@ -13508,11 +13508,11 @@
       <c r="C5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="256">
+      <c r="D5" s="268">
         <f>'CO_Attainment for Unit Tests'!C4</f>
         <v>314318</v>
       </c>
-      <c r="E5" s="208"/>
+      <c r="E5" s="209"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -13536,11 +13536,11 @@
       <c r="C6" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D6" s="256" t="str">
+      <c r="D6" s="268" t="str">
         <f>'CO_Attainment for Unit Tests'!C5</f>
         <v>4th Sem Co4K K-Scheme</v>
       </c>
-      <c r="E6" s="208"/>
+      <c r="E6" s="209"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
@@ -13564,11 +13564,11 @@
       <c r="C7" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="256" t="str">
+      <c r="D7" s="268" t="str">
         <f>'CO_Attainment for Unit Tests'!C6</f>
         <v>2024-25</v>
       </c>
-      <c r="E7" s="208"/>
+      <c r="E7" s="209"/>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
@@ -13591,41 +13591,41 @@
       <c r="E8" s="10"/>
     </row>
     <row r="9" spans="2:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="257" t="s">
+      <c r="B9" s="276" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="258" t="s">
+      <c r="C9" s="271" t="s">
         <v>56</v>
       </c>
-      <c r="D9" s="220" t="s">
+      <c r="D9" s="262" t="s">
         <v>57</v>
       </c>
-      <c r="E9" s="258" t="s">
+      <c r="E9" s="271" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B10" s="216"/>
-      <c r="C10" s="216"/>
-      <c r="D10" s="216"/>
-      <c r="E10" s="216"/>
+      <c r="B10" s="248"/>
+      <c r="C10" s="248"/>
+      <c r="D10" s="248"/>
+      <c r="E10" s="248"/>
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B11" s="216"/>
-      <c r="C11" s="216"/>
-      <c r="D11" s="216"/>
-      <c r="E11" s="216"/>
+      <c r="B11" s="248"/>
+      <c r="C11" s="248"/>
+      <c r="D11" s="248"/>
+      <c r="E11" s="248"/>
     </row>
     <row r="12" spans="2:22" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="216"/>
-      <c r="C12" s="216"/>
-      <c r="D12" s="216"/>
-      <c r="E12" s="217"/>
+      <c r="B12" s="248"/>
+      <c r="C12" s="248"/>
+      <c r="D12" s="248"/>
+      <c r="E12" s="249"/>
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B13" s="217"/>
-      <c r="C13" s="217"/>
-      <c r="D13" s="217"/>
+      <c r="B13" s="249"/>
+      <c r="C13" s="249"/>
+      <c r="D13" s="249"/>
       <c r="E13" s="55">
         <v>70</v>
       </c>
@@ -14928,7 +14928,7 @@
       <c r="D97" s="60" t="s">
         <v>152</v>
       </c>
-      <c r="E97" s="265">
+      <c r="E97" s="272">
         <f>D98*E13/100</f>
         <v>32.878999999999998</v>
       </c>
@@ -14937,7 +14937,7 @@
       <c r="D98" s="61">
         <v>46.97</v>
       </c>
-      <c r="E98" s="192"/>
+      <c r="E98" s="212"/>
     </row>
     <row r="99" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D99" s="62" t="s">
@@ -14963,11 +14963,11 @@
       <c r="E102" s="10"/>
     </row>
     <row r="103" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A103" s="229" t="s">
+      <c r="A103" s="236" t="s">
         <v>139</v>
       </c>
-      <c r="B103" s="200"/>
-      <c r="C103" s="200"/>
+      <c r="B103" s="203"/>
+      <c r="C103" s="203"/>
       <c r="D103" s="201"/>
       <c r="E103" s="66" t="s">
         <v>140</v>
@@ -14980,17 +14980,17 @@
       <c r="I103" s="68"/>
     </row>
     <row r="104" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="232" t="s">
+      <c r="A104" s="239" t="s">
         <v>142</v>
       </c>
       <c r="B104" s="69">
         <v>0.5</v>
       </c>
-      <c r="C104" s="266" t="s">
+      <c r="C104" s="273" t="s">
         <v>154</v>
       </c>
-      <c r="D104" s="267"/>
-      <c r="E104" s="268">
+      <c r="D104" s="274"/>
+      <c r="E104" s="275">
         <f>COUNTA(D14:D96)-COUNTIFS(D14:D96,0)</f>
         <v>70</v>
       </c>
@@ -15005,15 +15005,15 @@
       <c r="I104" s="68"/>
     </row>
     <row r="105" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="233"/>
+      <c r="A105" s="240"/>
       <c r="B105" s="72">
         <v>0.6</v>
       </c>
-      <c r="C105" s="259" t="s">
+      <c r="C105" s="277" t="s">
         <v>154</v>
       </c>
-      <c r="D105" s="254"/>
-      <c r="E105" s="191"/>
+      <c r="D105" s="246"/>
+      <c r="E105" s="211"/>
       <c r="F105" s="73">
         <f t="shared" si="0"/>
         <v>42</v>
@@ -15025,15 +15025,15 @@
       <c r="I105" s="68"/>
     </row>
     <row r="106" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A106" s="234"/>
+      <c r="A106" s="241"/>
       <c r="B106" s="75">
         <v>0.7</v>
       </c>
-      <c r="C106" s="260" t="s">
+      <c r="C106" s="278" t="s">
         <v>155</v>
       </c>
-      <c r="D106" s="227"/>
-      <c r="E106" s="192"/>
+      <c r="D106" s="234"/>
+      <c r="E106" s="212"/>
       <c r="F106" s="76">
         <f t="shared" si="0"/>
         <v>49</v>
@@ -15067,10 +15067,10 @@
       <c r="I108" s="68"/>
     </row>
     <row r="109" spans="1:9" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="261" t="s">
+      <c r="A109" s="279" t="s">
         <v>156</v>
       </c>
-      <c r="B109" s="262"/>
+      <c r="B109" s="280"/>
       <c r="C109" s="50" t="s">
         <v>9</v>
       </c>
@@ -15092,10 +15092,10 @@
       <c r="I109" s="68"/>
     </row>
     <row r="110" spans="1:9" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="263" t="s">
+      <c r="A110" s="269" t="s">
         <v>157</v>
       </c>
-      <c r="B110" s="264"/>
+      <c r="B110" s="270"/>
       <c r="C110" s="53">
         <f>IF(E99&gt;=$F106,3,IF(E99&gt;=$F105,2,IF(E99&gt;=$F104,1,0)))</f>
         <v>3</v>
@@ -16508,11 +16508,11 @@
       <c r="C4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="241" t="str">
+      <c r="D4" s="252" t="str">
         <f>'CO_Attainment for Unit Tests'!C3</f>
         <v>Data Communication and Computer Network (DCN)</v>
       </c>
-      <c r="E4" s="189"/>
+      <c r="E4" s="226"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
@@ -16522,11 +16522,11 @@
       <c r="C5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="241">
+      <c r="D5" s="252">
         <f>'CO_Attainment for Unit Tests'!C4</f>
         <v>314318</v>
       </c>
-      <c r="E5" s="189"/>
+      <c r="E5" s="226"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -16536,11 +16536,11 @@
       <c r="C6" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D6" s="241" t="str">
+      <c r="D6" s="252" t="str">
         <f>'CO_Attainment for Unit Tests'!C5</f>
         <v>4th Sem Co4K K-Scheme</v>
       </c>
-      <c r="E6" s="189"/>
+      <c r="E6" s="226"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
@@ -16550,63 +16550,63 @@
       <c r="C7" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="D7" s="241" t="str">
+      <c r="D7" s="252" t="str">
         <f>'CO_Attainment for Unit Tests'!C6</f>
         <v>2024-25</v>
       </c>
-      <c r="E7" s="189"/>
+      <c r="E7" s="226"/>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
     </row>
     <row r="9" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="257" t="s">
+      <c r="B9" s="276" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="258" t="s">
+      <c r="C9" s="271" t="s">
         <v>56</v>
       </c>
-      <c r="D9" s="269" t="s">
+      <c r="D9" s="281" t="s">
         <v>57</v>
       </c>
-      <c r="E9" s="258" t="s">
+      <c r="E9" s="271" t="s">
         <v>162</v>
       </c>
-      <c r="F9" s="258" t="s">
+      <c r="F9" s="271" t="s">
         <v>163</v>
       </c>
-      <c r="G9" s="258" t="s">
+      <c r="G9" s="271" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="10" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="216"/>
-      <c r="C10" s="216"/>
-      <c r="D10" s="216"/>
-      <c r="E10" s="216"/>
-      <c r="F10" s="216"/>
-      <c r="G10" s="216"/>
+      <c r="B10" s="248"/>
+      <c r="C10" s="248"/>
+      <c r="D10" s="248"/>
+      <c r="E10" s="248"/>
+      <c r="F10" s="248"/>
+      <c r="G10" s="248"/>
     </row>
     <row r="11" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="216"/>
-      <c r="C11" s="216"/>
-      <c r="D11" s="216"/>
-      <c r="E11" s="216"/>
-      <c r="F11" s="216"/>
-      <c r="G11" s="216"/>
+      <c r="B11" s="248"/>
+      <c r="C11" s="248"/>
+      <c r="D11" s="248"/>
+      <c r="E11" s="248"/>
+      <c r="F11" s="248"/>
+      <c r="G11" s="248"/>
     </row>
     <row r="12" spans="2:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="216"/>
-      <c r="C12" s="216"/>
-      <c r="D12" s="216"/>
-      <c r="E12" s="217"/>
-      <c r="F12" s="217"/>
-      <c r="G12" s="217"/>
+      <c r="B12" s="248"/>
+      <c r="C12" s="248"/>
+      <c r="D12" s="248"/>
+      <c r="E12" s="249"/>
+      <c r="F12" s="249"/>
+      <c r="G12" s="249"/>
     </row>
     <row r="13" spans="2:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="217"/>
-      <c r="C13" s="217"/>
-      <c r="D13" s="217"/>
+      <c r="B13" s="249"/>
+      <c r="C13" s="249"/>
+      <c r="D13" s="249"/>
       <c r="E13" s="29">
         <v>25</v>
       </c>
@@ -16832,7 +16832,7 @@
       </c>
       <c r="F23" s="58"/>
       <c r="G23" s="58"/>
-      <c r="H23" s="336"/>
+      <c r="H23" s="198"/>
     </row>
     <row r="24" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="56">
@@ -17115,7 +17115,7 @@
       </c>
       <c r="F36" s="58"/>
       <c r="G36" s="58"/>
-      <c r="H36" s="337"/>
+      <c r="H36" s="199"/>
     </row>
     <row r="37" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="56">
@@ -17464,7 +17464,7 @@
       </c>
       <c r="F52" s="58"/>
       <c r="G52" s="58"/>
-      <c r="H52" s="337"/>
+      <c r="H52" s="199"/>
     </row>
     <row r="53" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="56">
@@ -17483,7 +17483,7 @@
       </c>
       <c r="F53" s="58"/>
       <c r="G53" s="58"/>
-      <c r="H53" s="337"/>
+      <c r="H53" s="199"/>
     </row>
     <row r="54" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="56">
@@ -17720,7 +17720,7 @@
       <c r="E64" s="58"/>
       <c r="F64" s="58"/>
       <c r="G64" s="58"/>
-      <c r="H64" s="337"/>
+      <c r="H64" s="199"/>
     </row>
     <row r="65" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B65" s="56">
@@ -18354,15 +18354,15 @@
       <c r="D97" s="81" t="s">
         <v>165</v>
       </c>
-      <c r="E97" s="270">
+      <c r="E97" s="283">
         <f>ROUNDUP(D98*E13/100,1)</f>
         <v>15</v>
       </c>
-      <c r="F97" s="270">
+      <c r="F97" s="283">
         <f>ROUNDUP(D98*F13/100,1)</f>
         <v>15</v>
       </c>
-      <c r="G97" s="270">
+      <c r="G97" s="283">
         <f>ROUNDUP(D98*G13/100,1)</f>
         <v>15</v>
       </c>
@@ -18371,9 +18371,9 @@
       <c r="D98" s="82">
         <v>60</v>
       </c>
-      <c r="E98" s="192"/>
-      <c r="F98" s="192"/>
-      <c r="G98" s="192"/>
+      <c r="E98" s="212"/>
+      <c r="F98" s="212"/>
+      <c r="G98" s="212"/>
     </row>
     <row r="99" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D99" s="62" t="s">
@@ -18397,10 +18397,10 @@
     <row r="102" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="103" spans="1:8" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="68"/>
-      <c r="B103" s="229" t="s">
+      <c r="B103" s="236" t="s">
         <v>166</v>
       </c>
-      <c r="C103" s="200"/>
+      <c r="C103" s="203"/>
       <c r="D103" s="201"/>
       <c r="E103" s="83" t="s">
         <v>140</v>
@@ -18413,7 +18413,7 @@
     </row>
     <row r="104" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="68"/>
-      <c r="B104" s="232" t="s">
+      <c r="B104" s="239" t="s">
         <v>142</v>
       </c>
       <c r="C104" s="84">
@@ -18422,7 +18422,7 @@
       <c r="D104" s="70" t="s">
         <v>155</v>
       </c>
-      <c r="E104" s="268">
+      <c r="E104" s="275">
         <f>COUNTA(D14:D96)-COUNTIFS(D14:D96,0)</f>
         <v>70</v>
       </c>
@@ -18437,14 +18437,14 @@
     </row>
     <row r="105" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="68"/>
-      <c r="B105" s="233"/>
+      <c r="B105" s="240"/>
       <c r="C105" s="86">
         <v>0.6</v>
       </c>
       <c r="D105" s="73" t="s">
         <v>155</v>
       </c>
-      <c r="E105" s="191"/>
+      <c r="E105" s="211"/>
       <c r="F105" s="87">
         <f>C105*$E104</f>
         <v>42</v>
@@ -18456,14 +18456,14 @@
     </row>
     <row r="106" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="68"/>
-      <c r="B106" s="234"/>
+      <c r="B106" s="241"/>
       <c r="C106" s="88">
         <v>0.7</v>
       </c>
       <c r="D106" s="76" t="s">
         <v>155</v>
       </c>
-      <c r="E106" s="192"/>
+      <c r="E106" s="212"/>
       <c r="F106" s="89">
         <f>C106*$E104</f>
         <v>49</v>
@@ -18494,10 +18494,10 @@
       <c r="H108" s="68"/>
     </row>
     <row r="109" spans="1:8" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="199" t="s">
+      <c r="A109" s="200" t="s">
         <v>167</v>
       </c>
-      <c r="B109" s="271"/>
+      <c r="B109" s="284"/>
       <c r="C109" s="90" t="s">
         <v>9</v>
       </c>
@@ -18518,10 +18518,10 @@
       </c>
     </row>
     <row r="110" spans="1:8" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="272" t="s">
+      <c r="A110" s="285" t="s">
         <v>168</v>
       </c>
-      <c r="B110" s="262"/>
+      <c r="B110" s="280"/>
       <c r="C110" s="92">
         <f>IF(E99&gt;=$F106,3,IF(E99&gt;=$F105,2,IF(E99&gt;=$F104,1,0)))</f>
         <v>3</v>
@@ -18548,10 +18548,10 @@
       </c>
     </row>
     <row r="111" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A111" s="273" t="s">
+      <c r="A111" s="286" t="s">
         <v>169</v>
       </c>
-      <c r="B111" s="189"/>
+      <c r="B111" s="226"/>
       <c r="C111" s="94">
         <f>IF(F99&gt;=$F106,3,IF(F99&gt;=$F105,2,IF(F99&gt;=$F104,1,0)))</f>
         <v>3</v>
@@ -18578,10 +18578,10 @@
       </c>
     </row>
     <row r="112" spans="1:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A112" s="274" t="s">
+      <c r="A112" s="282" t="s">
         <v>170</v>
       </c>
-      <c r="B112" s="264"/>
+      <c r="B112" s="270"/>
       <c r="C112" s="53">
         <f>IF(G99&gt;=$F106,3,IF(G99&gt;=$F105,2,IF(G99&gt;=$F104,1,0)))</f>
         <v>3</v>
@@ -19628,41 +19628,41 @@
       </c>
     </row>
     <row r="10" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="281" t="s">
+      <c r="B10" s="289" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="282" t="s">
+      <c r="C10" s="290" t="s">
         <v>173</v>
       </c>
-      <c r="D10" s="283" t="s">
+      <c r="D10" s="291" t="s">
         <v>57</v>
       </c>
-      <c r="E10" s="282" t="s">
+      <c r="E10" s="290" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B11" s="191"/>
-      <c r="C11" s="191"/>
-      <c r="D11" s="191"/>
-      <c r="E11" s="191"/>
+      <c r="B11" s="211"/>
+      <c r="C11" s="211"/>
+      <c r="D11" s="211"/>
+      <c r="E11" s="211"/>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B12" s="191"/>
-      <c r="C12" s="191"/>
-      <c r="D12" s="191"/>
-      <c r="E12" s="191"/>
+      <c r="B12" s="211"/>
+      <c r="C12" s="211"/>
+      <c r="D12" s="211"/>
+      <c r="E12" s="211"/>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B13" s="191"/>
-      <c r="C13" s="191"/>
-      <c r="D13" s="191"/>
-      <c r="E13" s="284"/>
+      <c r="B13" s="211"/>
+      <c r="C13" s="211"/>
+      <c r="D13" s="211"/>
+      <c r="E13" s="292"/>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="192"/>
-      <c r="C14" s="192"/>
-      <c r="D14" s="192"/>
+      <c r="B14" s="212"/>
+      <c r="C14" s="212"/>
+      <c r="D14" s="212"/>
       <c r="E14" s="99">
         <v>5</v>
       </c>
@@ -20459,57 +20459,57 @@
     </row>
     <row r="84" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="85" spans="1:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="285" t="s">
+      <c r="A85" s="293" t="s">
         <v>179</v>
       </c>
-      <c r="B85" s="200"/>
-      <c r="C85" s="200"/>
+      <c r="B85" s="203"/>
+      <c r="C85" s="203"/>
       <c r="D85" s="201"/>
       <c r="E85" s="106" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="86" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="286" t="s">
+      <c r="A86" s="294" t="s">
         <v>142</v>
       </c>
-      <c r="B86" s="287" t="s">
+      <c r="B86" s="295" t="s">
         <v>180</v>
       </c>
-      <c r="C86" s="288"/>
-      <c r="D86" s="267"/>
+      <c r="C86" s="296"/>
+      <c r="D86" s="274"/>
       <c r="E86" s="107">
         <v>1</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="233"/>
-      <c r="B87" s="275" t="s">
+      <c r="A87" s="240"/>
+      <c r="B87" s="297" t="s">
         <v>181</v>
       </c>
-      <c r="C87" s="276"/>
-      <c r="D87" s="254"/>
+      <c r="C87" s="298"/>
+      <c r="D87" s="246"/>
       <c r="E87" s="108">
         <v>2</v>
       </c>
     </row>
     <row r="88" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="234"/>
-      <c r="B88" s="277" t="s">
+      <c r="A88" s="241"/>
+      <c r="B88" s="299" t="s">
         <v>182</v>
       </c>
-      <c r="C88" s="278"/>
-      <c r="D88" s="227"/>
+      <c r="C88" s="300"/>
+      <c r="D88" s="234"/>
       <c r="E88" s="109">
         <v>3</v>
       </c>
     </row>
     <row r="89" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="90" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="279" t="s">
+      <c r="A90" s="287" t="s">
         <v>167</v>
       </c>
-      <c r="B90" s="271"/>
+      <c r="B90" s="284"/>
       <c r="C90" s="110" t="s">
         <v>9</v>
       </c>
@@ -20527,10 +20527,10 @@
       </c>
     </row>
     <row r="91" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="280" t="s">
+      <c r="A91" s="288" t="s">
         <v>183</v>
       </c>
-      <c r="B91" s="262"/>
+      <c r="B91" s="280"/>
       <c r="C91" s="112">
         <f>IF(E81&gt;=80,3,IF(E81&gt;=65,2,IF(E81&gt;=40,1,0)))</f>
         <v>0</v>
@@ -21547,34 +21547,34 @@
       <c r="P5" s="10"/>
     </row>
     <row r="6" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B6" s="190" t="s">
+      <c r="B6" s="210" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="193" t="s">
+      <c r="C6" s="213" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="194"/>
-      <c r="E6" s="199" t="s">
+      <c r="D6" s="214"/>
+      <c r="E6" s="200" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="200"/>
-      <c r="G6" s="200"/>
-      <c r="H6" s="200"/>
-      <c r="I6" s="200"/>
-      <c r="J6" s="200"/>
-      <c r="K6" s="200"/>
-      <c r="L6" s="200"/>
-      <c r="M6" s="200"/>
+      <c r="F6" s="203"/>
+      <c r="G6" s="203"/>
+      <c r="H6" s="203"/>
+      <c r="I6" s="203"/>
+      <c r="J6" s="203"/>
+      <c r="K6" s="203"/>
+      <c r="L6" s="203"/>
+      <c r="M6" s="203"/>
       <c r="N6" s="201"/>
-      <c r="O6" s="199" t="s">
+      <c r="O6" s="200" t="s">
         <v>24</v>
       </c>
       <c r="P6" s="201"/>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B7" s="191"/>
-      <c r="C7" s="195"/>
-      <c r="D7" s="196"/>
+      <c r="B7" s="211"/>
+      <c r="C7" s="215"/>
+      <c r="D7" s="216"/>
       <c r="E7" s="13" t="s">
         <v>25</v>
       </c>
@@ -21613,9 +21613,9 @@
       </c>
     </row>
     <row r="8" spans="2:16" ht="62.25" x14ac:dyDescent="0.25">
-      <c r="B8" s="192"/>
-      <c r="C8" s="197"/>
-      <c r="D8" s="198"/>
+      <c r="B8" s="212"/>
+      <c r="C8" s="217"/>
+      <c r="D8" s="218"/>
       <c r="E8" s="14" t="s">
         <v>192</v>
       </c>
@@ -21936,10 +21936,10 @@
       </c>
     </row>
     <row r="15" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B15" s="289" t="s">
+      <c r="B15" s="301" t="s">
         <v>211</v>
       </c>
-      <c r="C15" s="200"/>
+      <c r="C15" s="203"/>
       <c r="D15" s="201"/>
       <c r="E15" s="119">
         <f t="shared" ref="E15:P15" si="0">ROUNDUP(AVERAGE(E9:E14),2)</f>
@@ -21991,10 +21991,10 @@
       </c>
     </row>
     <row r="16" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B16" s="290" t="s">
+      <c r="B16" s="302" t="s">
         <v>212</v>
       </c>
-      <c r="C16" s="200"/>
+      <c r="C16" s="203"/>
       <c r="D16" s="201"/>
       <c r="E16" s="120">
         <f t="shared" ref="E16:P16" si="1">ROUNDUP((E15*2.66)/3,2)</f>
@@ -22046,10 +22046,10 @@
       </c>
     </row>
     <row r="17" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B17" s="290" t="s">
+      <c r="B17" s="302" t="s">
         <v>213</v>
       </c>
-      <c r="C17" s="200"/>
+      <c r="C17" s="203"/>
       <c r="D17" s="201"/>
       <c r="E17" s="120">
         <f t="shared" ref="E17:P17" si="2">ROUNDUP((E16/3)*100,2)</f>
@@ -23082,13 +23082,13 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="O6:P6"/>
+    <mergeCell ref="B15:D15"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="C6:D8"/>
     <mergeCell ref="E6:N6"/>
-    <mergeCell ref="O6:P6"/>
-    <mergeCell ref="B15:D15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -23337,15 +23337,15 @@
     <row r="8" spans="1:26" ht="21" x14ac:dyDescent="0.25">
       <c r="A8" s="10"/>
       <c r="B8" s="10"/>
-      <c r="C8" s="291" t="s">
+      <c r="C8" s="303" t="s">
         <v>215</v>
       </c>
-      <c r="D8" s="200"/>
-      <c r="E8" s="200"/>
-      <c r="F8" s="200"/>
-      <c r="G8" s="200"/>
-      <c r="H8" s="200"/>
-      <c r="I8" s="200"/>
+      <c r="D8" s="203"/>
+      <c r="E8" s="203"/>
+      <c r="F8" s="203"/>
+      <c r="G8" s="203"/>
+      <c r="H8" s="203"/>
+      <c r="I8" s="203"/>
       <c r="J8" s="201"/>
       <c r="K8" s="10"/>
       <c r="L8" s="10"/>
@@ -23367,18 +23367,18 @@
     <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" s="10"/>
       <c r="B9" s="10"/>
-      <c r="C9" s="292" t="s">
+      <c r="C9" s="304" t="s">
         <v>216</v>
       </c>
-      <c r="D9" s="200"/>
-      <c r="E9" s="200"/>
-      <c r="F9" s="200"/>
-      <c r="G9" s="200"/>
+      <c r="D9" s="203"/>
+      <c r="E9" s="203"/>
+      <c r="F9" s="203"/>
+      <c r="G9" s="203"/>
       <c r="H9" s="201"/>
-      <c r="I9" s="293" t="s">
+      <c r="I9" s="305" t="s">
         <v>217</v>
       </c>
-      <c r="J9" s="194"/>
+      <c r="J9" s="214"/>
       <c r="K9" s="10"/>
       <c r="L9" s="10"/>
       <c r="M9" s="10"/>
@@ -23399,20 +23399,20 @@
     <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" s="10"/>
       <c r="B10" s="10"/>
-      <c r="C10" s="294" t="s">
+      <c r="C10" s="306" t="s">
         <v>218</v>
       </c>
-      <c r="D10" s="295" t="s">
+      <c r="D10" s="307" t="s">
         <v>219</v>
       </c>
-      <c r="E10" s="296"/>
-      <c r="F10" s="296"/>
-      <c r="G10" s="198"/>
+      <c r="E10" s="308"/>
+      <c r="F10" s="308"/>
+      <c r="G10" s="218"/>
       <c r="H10" s="122" t="s">
         <v>220</v>
       </c>
-      <c r="I10" s="197"/>
-      <c r="J10" s="198"/>
+      <c r="I10" s="217"/>
+      <c r="J10" s="218"/>
       <c r="K10" s="10"/>
       <c r="L10" s="10"/>
       <c r="M10" s="10"/>
@@ -23433,7 +23433,7 @@
     <row r="11" spans="1:26" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10"/>
       <c r="B11" s="10"/>
-      <c r="C11" s="192"/>
+      <c r="C11" s="212"/>
       <c r="D11" s="123" t="s">
         <v>221</v>
       </c>
@@ -23449,7 +23449,7 @@
       <c r="H11" s="126" t="s">
         <v>225</v>
       </c>
-      <c r="I11" s="297" t="s">
+      <c r="I11" s="309" t="s">
         <v>226</v>
       </c>
       <c r="J11" s="201"/>
@@ -23496,11 +23496,11 @@
         <f>'CO_attainment for FA-TH ESE'!C110</f>
         <v>3</v>
       </c>
-      <c r="I12" s="298">
+      <c r="I12" s="310">
         <f>'CO_attainment for Indirect'!C91</f>
         <v>0</v>
       </c>
-      <c r="J12" s="267"/>
+      <c r="J12" s="274"/>
       <c r="K12" s="10"/>
       <c r="L12" s="10"/>
       <c r="M12" s="10"/>
@@ -23544,11 +23544,11 @@
         <f t="shared" ref="H13:H17" si="3">$H12</f>
         <v>3</v>
       </c>
-      <c r="I13" s="302">
+      <c r="I13" s="314">
         <f t="shared" ref="I13:I17" si="4">$I12</f>
         <v>0</v>
       </c>
-      <c r="J13" s="254"/>
+      <c r="J13" s="246"/>
       <c r="K13" s="10"/>
       <c r="L13" s="10"/>
       <c r="M13" s="10"/>
@@ -23592,11 +23592,11 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="I14" s="302">
+      <c r="I14" s="314">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="J14" s="254"/>
+      <c r="J14" s="246"/>
       <c r="K14" s="10"/>
       <c r="L14" s="10"/>
       <c r="M14" s="10"/>
@@ -23640,11 +23640,11 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="I15" s="302">
+      <c r="I15" s="314">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="J15" s="254"/>
+      <c r="J15" s="246"/>
       <c r="K15" s="10"/>
       <c r="L15" s="10"/>
       <c r="M15" s="10"/>
@@ -23688,11 +23688,11 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="I16" s="302">
+      <c r="I16" s="314">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="J16" s="254"/>
+      <c r="J16" s="246"/>
       <c r="K16" s="10"/>
       <c r="L16" s="10"/>
       <c r="M16" s="10"/>
@@ -23736,11 +23736,11 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="I17" s="302">
+      <c r="I17" s="314">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="J17" s="254"/>
+      <c r="J17" s="246"/>
       <c r="K17" s="10"/>
       <c r="L17" s="10"/>
       <c r="M17" s="10"/>
@@ -23784,11 +23784,11 @@
         <f t="shared" si="5"/>
         <v>3</v>
       </c>
-      <c r="I18" s="298">
+      <c r="I18" s="310">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="J18" s="267"/>
+      <c r="J18" s="274"/>
       <c r="K18" s="10"/>
       <c r="L18" s="10"/>
       <c r="M18" s="10"/>
@@ -23827,10 +23827,10 @@
       <c r="H19" s="140">
         <v>60</v>
       </c>
-      <c r="I19" s="303">
+      <c r="I19" s="315">
         <v>100</v>
       </c>
-      <c r="J19" s="189"/>
+      <c r="J19" s="226"/>
       <c r="K19" s="10"/>
       <c r="L19" s="10"/>
       <c r="M19" s="10"/>
@@ -23874,11 +23874,11 @@
         <f t="shared" si="6"/>
         <v>1.8</v>
       </c>
-      <c r="I20" s="299">
+      <c r="I20" s="311">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="J20" s="227"/>
+      <c r="J20" s="234"/>
       <c r="K20" s="10"/>
       <c r="L20" s="10"/>
       <c r="M20" s="10"/>
@@ -23899,12 +23899,12 @@
     <row r="21" spans="1:26" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="10"/>
       <c r="B21" s="10"/>
-      <c r="C21" s="300" t="s">
+      <c r="C21" s="312" t="s">
         <v>230</v>
       </c>
-      <c r="D21" s="200"/>
-      <c r="E21" s="200"/>
-      <c r="F21" s="200"/>
+      <c r="D21" s="203"/>
+      <c r="E21" s="203"/>
+      <c r="F21" s="203"/>
       <c r="G21" s="201"/>
       <c r="H21" s="142">
         <f>SUM(D20:H20)</f>
@@ -23937,12 +23937,12 @@
     <row r="22" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="10"/>
       <c r="B22" s="10"/>
-      <c r="C22" s="300" t="s">
+      <c r="C22" s="312" t="s">
         <v>232</v>
       </c>
-      <c r="D22" s="200"/>
-      <c r="E22" s="200"/>
-      <c r="F22" s="200"/>
+      <c r="D22" s="203"/>
+      <c r="E22" s="203"/>
+      <c r="F22" s="203"/>
       <c r="G22" s="201"/>
       <c r="H22" s="144">
         <v>0.8</v>
@@ -23973,12 +23973,12 @@
     <row r="23" spans="1:26" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="10"/>
       <c r="B23" s="10"/>
-      <c r="C23" s="300" t="s">
+      <c r="C23" s="312" t="s">
         <v>234</v>
       </c>
-      <c r="D23" s="200"/>
-      <c r="E23" s="200"/>
-      <c r="F23" s="200"/>
+      <c r="D23" s="203"/>
+      <c r="E23" s="203"/>
+      <c r="F23" s="203"/>
       <c r="G23" s="201"/>
       <c r="H23" s="142">
         <f>0.8*H21</f>
@@ -24011,13 +24011,13 @@
     <row r="24" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="10"/>
       <c r="B24" s="10"/>
-      <c r="C24" s="301" t="s">
+      <c r="C24" s="313" t="s">
         <v>236</v>
       </c>
-      <c r="D24" s="200"/>
-      <c r="E24" s="200"/>
-      <c r="F24" s="200"/>
-      <c r="G24" s="200"/>
+      <c r="D24" s="203"/>
+      <c r="E24" s="203"/>
+      <c r="F24" s="203"/>
+      <c r="G24" s="203"/>
       <c r="H24" s="201"/>
       <c r="I24" s="146">
         <f>ROUNDUP(H23+J23,2)</f>
@@ -30880,15 +30880,15 @@
     <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" s="10"/>
       <c r="B8" s="6"/>
-      <c r="C8" s="304" t="s">
+      <c r="C8" s="316" t="s">
         <v>239</v>
       </c>
-      <c r="D8" s="305"/>
-      <c r="E8" s="307" t="s">
+      <c r="D8" s="317"/>
+      <c r="E8" s="319" t="s">
         <v>240</v>
       </c>
-      <c r="F8" s="288"/>
-      <c r="G8" s="262"/>
+      <c r="F8" s="296"/>
+      <c r="G8" s="280"/>
       <c r="H8" s="148" t="s">
         <v>241</v>
       </c>
@@ -30898,7 +30898,7 @@
       <c r="J8" s="148" t="s">
         <v>243</v>
       </c>
-      <c r="K8" s="308" t="s">
+      <c r="K8" s="320" t="s">
         <v>244</v>
       </c>
       <c r="L8" s="10"/>
@@ -30920,8 +30920,8 @@
     <row r="9" spans="1:26" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="10"/>
       <c r="B9" s="6"/>
-      <c r="C9" s="197"/>
-      <c r="D9" s="306"/>
+      <c r="C9" s="217"/>
+      <c r="D9" s="318"/>
       <c r="E9" s="149" t="s">
         <v>245</v>
       </c>
@@ -30940,7 +30940,7 @@
       <c r="J9" s="150" t="s">
         <v>225</v>
       </c>
-      <c r="K9" s="309"/>
+      <c r="K9" s="321"/>
       <c r="L9" s="10"/>
       <c r="M9" s="10"/>
       <c r="N9" s="10"/>
@@ -30960,14 +30960,14 @@
     <row r="10" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="10"/>
       <c r="B10" s="6"/>
-      <c r="C10" s="310" t="s">
+      <c r="C10" s="322" t="s">
         <v>249</v>
       </c>
-      <c r="D10" s="262"/>
-      <c r="E10" s="311">
+      <c r="D10" s="280"/>
+      <c r="E10" s="323">
         <v>30</v>
       </c>
-      <c r="F10" s="262"/>
+      <c r="F10" s="280"/>
       <c r="G10" s="151">
         <v>25</v>
       </c>
@@ -31003,15 +31003,15 @@
     <row r="11" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10"/>
       <c r="B11" s="6"/>
-      <c r="C11" s="312" t="s">
+      <c r="C11" s="324" t="s">
         <v>250</v>
       </c>
-      <c r="D11" s="264"/>
-      <c r="E11" s="313">
+      <c r="D11" s="270"/>
+      <c r="E11" s="325">
         <f>(E10/$K10)*100</f>
         <v>17.142857142857142</v>
       </c>
-      <c r="F11" s="264"/>
+      <c r="F11" s="270"/>
       <c r="G11" s="152">
         <f t="shared" ref="G11:J11" si="1">(G10/$K10)*100</f>
         <v>14.285714285714285</v>
@@ -31135,15 +31135,15 @@
     <row r="15" spans="1:26" ht="21" x14ac:dyDescent="0.25">
       <c r="A15" s="10"/>
       <c r="B15" s="10"/>
-      <c r="C15" s="314" t="s">
+      <c r="C15" s="326" t="s">
         <v>215</v>
       </c>
-      <c r="D15" s="200"/>
-      <c r="E15" s="200"/>
-      <c r="F15" s="200"/>
-      <c r="G15" s="200"/>
-      <c r="H15" s="200"/>
-      <c r="I15" s="200"/>
+      <c r="D15" s="203"/>
+      <c r="E15" s="203"/>
+      <c r="F15" s="203"/>
+      <c r="G15" s="203"/>
+      <c r="H15" s="203"/>
+      <c r="I15" s="203"/>
       <c r="J15" s="201"/>
       <c r="K15" s="10"/>
       <c r="L15" s="10"/>
@@ -31165,16 +31165,16 @@
     <row r="16" spans="1:26" ht="21" x14ac:dyDescent="0.25">
       <c r="A16" s="10"/>
       <c r="B16" s="10"/>
-      <c r="C16" s="315" t="s">
+      <c r="C16" s="327" t="s">
         <v>216</v>
       </c>
-      <c r="D16" s="200"/>
-      <c r="E16" s="200"/>
-      <c r="F16" s="200"/>
-      <c r="G16" s="200"/>
+      <c r="D16" s="203"/>
+      <c r="E16" s="203"/>
+      <c r="F16" s="203"/>
+      <c r="G16" s="203"/>
       <c r="H16" s="201"/>
-      <c r="I16" s="316"/>
-      <c r="J16" s="194"/>
+      <c r="I16" s="328"/>
+      <c r="J16" s="214"/>
       <c r="K16" s="10"/>
       <c r="L16" s="10"/>
       <c r="M16" s="10"/>
@@ -31195,7 +31195,7 @@
     <row r="17" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A17" s="10"/>
       <c r="B17" s="10"/>
-      <c r="C17" s="317" t="s">
+      <c r="C17" s="329" t="s">
         <v>251</v>
       </c>
       <c r="D17" s="154"/>
@@ -31207,8 +31207,8 @@
       <c r="H17" s="158" t="s">
         <v>220</v>
       </c>
-      <c r="I17" s="197"/>
-      <c r="J17" s="198"/>
+      <c r="I17" s="217"/>
+      <c r="J17" s="218"/>
       <c r="K17" s="10"/>
       <c r="L17" s="10"/>
       <c r="M17" s="10"/>
@@ -31229,7 +31229,7 @@
     <row r="18" spans="1:26" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="10"/>
       <c r="B18" s="10"/>
-      <c r="C18" s="192"/>
+      <c r="C18" s="212"/>
       <c r="D18" s="159" t="s">
         <v>221</v>
       </c>
@@ -31245,7 +31245,7 @@
       <c r="H18" s="162" t="s">
         <v>225</v>
       </c>
-      <c r="I18" s="318"/>
+      <c r="I18" s="330"/>
       <c r="J18" s="201"/>
       <c r="K18" s="10"/>
       <c r="L18" s="10"/>
@@ -31290,8 +31290,8 @@
         <f>'CO_attainment for FA-TH ESE'!C110</f>
         <v>3</v>
       </c>
-      <c r="I19" s="319"/>
-      <c r="J19" s="267"/>
+      <c r="I19" s="331"/>
+      <c r="J19" s="274"/>
       <c r="K19" s="10"/>
       <c r="L19" s="10"/>
       <c r="M19" s="10"/>
@@ -31335,8 +31335,8 @@
         <f t="shared" ref="H20:H24" si="5">$H19</f>
         <v>3</v>
       </c>
-      <c r="I20" s="320"/>
-      <c r="J20" s="254"/>
+      <c r="I20" s="332"/>
+      <c r="J20" s="246"/>
       <c r="K20" s="10"/>
       <c r="L20" s="10"/>
       <c r="M20" s="10"/>
@@ -31380,8 +31380,8 @@
         <f t="shared" si="5"/>
         <v>3</v>
       </c>
-      <c r="I21" s="320"/>
-      <c r="J21" s="254"/>
+      <c r="I21" s="332"/>
+      <c r="J21" s="246"/>
       <c r="K21" s="10"/>
       <c r="L21" s="10"/>
       <c r="M21" s="10"/>
@@ -31425,8 +31425,8 @@
         <f t="shared" si="5"/>
         <v>3</v>
       </c>
-      <c r="I22" s="320"/>
-      <c r="J22" s="254"/>
+      <c r="I22" s="332"/>
+      <c r="J22" s="246"/>
       <c r="K22" s="10"/>
       <c r="L22" s="10"/>
       <c r="M22" s="10"/>
@@ -31470,8 +31470,8 @@
         <f t="shared" si="5"/>
         <v>3</v>
       </c>
-      <c r="I23" s="320"/>
-      <c r="J23" s="254"/>
+      <c r="I23" s="332"/>
+      <c r="J23" s="246"/>
       <c r="K23" s="10"/>
       <c r="L23" s="10"/>
       <c r="M23" s="10"/>
@@ -31515,8 +31515,8 @@
         <f t="shared" si="5"/>
         <v>3</v>
       </c>
-      <c r="I24" s="320"/>
-      <c r="J24" s="254"/>
+      <c r="I24" s="332"/>
+      <c r="J24" s="246"/>
       <c r="K24" s="10"/>
       <c r="L24" s="10"/>
       <c r="M24" s="10"/>
@@ -31560,8 +31560,8 @@
         <f t="shared" si="6"/>
         <v>3</v>
       </c>
-      <c r="I25" s="319"/>
-      <c r="J25" s="267"/>
+      <c r="I25" s="331"/>
+      <c r="J25" s="274"/>
       <c r="K25" s="10"/>
       <c r="L25" s="10"/>
       <c r="M25" s="10"/>
@@ -31605,8 +31605,8 @@
         <f t="shared" si="7"/>
         <v>40</v>
       </c>
-      <c r="I26" s="324"/>
-      <c r="J26" s="254"/>
+      <c r="I26" s="336"/>
+      <c r="J26" s="246"/>
       <c r="K26" s="10"/>
       <c r="L26" s="10"/>
       <c r="M26" s="10"/>
@@ -31650,8 +31650,8 @@
         <f t="shared" si="8"/>
         <v>1.2</v>
       </c>
-      <c r="I27" s="325"/>
-      <c r="J27" s="227"/>
+      <c r="I27" s="337"/>
+      <c r="J27" s="234"/>
       <c r="K27" s="10"/>
       <c r="L27" s="10"/>
       <c r="M27" s="10"/>
@@ -31672,12 +31672,12 @@
     <row r="28" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="10"/>
       <c r="B28" s="10"/>
-      <c r="C28" s="321" t="s">
+      <c r="C28" s="333" t="s">
         <v>230</v>
       </c>
-      <c r="D28" s="200"/>
-      <c r="E28" s="200"/>
-      <c r="F28" s="200"/>
+      <c r="D28" s="203"/>
+      <c r="E28" s="203"/>
+      <c r="F28" s="203"/>
       <c r="G28" s="201"/>
       <c r="H28" s="177">
         <f>SUM(D27:H27)</f>
@@ -31705,12 +31705,12 @@
     <row r="29" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="10"/>
       <c r="B29" s="10"/>
-      <c r="C29" s="321" t="s">
+      <c r="C29" s="333" t="s">
         <v>232</v>
       </c>
-      <c r="D29" s="200"/>
-      <c r="E29" s="200"/>
-      <c r="F29" s="200"/>
+      <c r="D29" s="203"/>
+      <c r="E29" s="203"/>
+      <c r="F29" s="203"/>
       <c r="G29" s="201"/>
       <c r="H29" s="180">
         <v>1</v>
@@ -31737,12 +31737,12 @@
     <row r="30" spans="1:26" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="10"/>
       <c r="B30" s="10"/>
-      <c r="C30" s="321" t="s">
+      <c r="C30" s="333" t="s">
         <v>234</v>
       </c>
-      <c r="D30" s="200"/>
-      <c r="E30" s="200"/>
-      <c r="F30" s="200"/>
+      <c r="D30" s="203"/>
+      <c r="E30" s="203"/>
+      <c r="F30" s="203"/>
       <c r="G30" s="201"/>
       <c r="H30" s="177">
         <f>H29*H28</f>
@@ -31770,13 +31770,13 @@
     <row r="31" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="10"/>
       <c r="B31" s="10"/>
-      <c r="C31" s="322" t="s">
+      <c r="C31" s="334" t="s">
         <v>236</v>
       </c>
-      <c r="D31" s="200"/>
-      <c r="E31" s="200"/>
-      <c r="F31" s="200"/>
-      <c r="G31" s="200"/>
+      <c r="D31" s="203"/>
+      <c r="E31" s="203"/>
+      <c r="F31" s="203"/>
+      <c r="G31" s="203"/>
       <c r="H31" s="201"/>
       <c r="I31" s="182">
         <f>H30+J30</f>
@@ -31864,11 +31864,11 @@
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
       <c r="G34" s="10"/>
-      <c r="H34" s="204" t="s">
+      <c r="H34" s="205" t="s">
         <v>47</v>
       </c>
-      <c r="I34" s="205"/>
-      <c r="J34" s="205"/>
+      <c r="I34" s="206"/>
+      <c r="J34" s="206"/>
       <c r="L34" s="10"/>
       <c r="M34" s="10"/>
       <c r="N34" s="10"/>
@@ -31893,11 +31893,11 @@
       <c r="E35" s="10"/>
       <c r="F35" s="10"/>
       <c r="G35" s="10"/>
-      <c r="H35" s="323" t="s">
+      <c r="H35" s="335" t="s">
         <v>48</v>
       </c>
-      <c r="I35" s="207"/>
-      <c r="J35" s="208"/>
+      <c r="I35" s="208"/>
+      <c r="J35" s="209"/>
       <c r="K35" s="11"/>
       <c r="L35" s="11"/>
       <c r="M35" s="11"/>
@@ -38373,11 +38373,11 @@
       <c r="C2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="241" t="str">
+      <c r="D2" s="252" t="str">
         <f>'Overall CO attainment'!D3</f>
         <v>Data Communication and Computer Network (DCN)</v>
       </c>
-      <c r="E2" s="189"/>
+      <c r="E2" s="226"/>
       <c r="F2" s="11"/>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
@@ -38405,11 +38405,11 @@
       <c r="C3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="241">
+      <c r="D3" s="252">
         <f>'Overall CO attainment'!D4</f>
         <v>314318</v>
       </c>
-      <c r="E3" s="189"/>
+      <c r="E3" s="226"/>
       <c r="F3" s="11"/>
       <c r="G3" s="11"/>
       <c r="H3" s="11"/>
@@ -38437,11 +38437,11 @@
       <c r="C4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="241" t="str">
+      <c r="D4" s="252" t="str">
         <f>'Overall CO attainment'!D5</f>
         <v>4th Sem Co4K K-Scheme</v>
       </c>
-      <c r="E4" s="189"/>
+      <c r="E4" s="226"/>
       <c r="F4" s="11"/>
       <c r="G4" s="11"/>
       <c r="H4" s="11"/>
@@ -38469,11 +38469,11 @@
       <c r="C5" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="D5" s="241" t="str">
+      <c r="D5" s="252" t="str">
         <f>'Overall CO attainment'!D6</f>
         <v>2024-25</v>
       </c>
-      <c r="E5" s="189"/>
+      <c r="E5" s="226"/>
       <c r="F5" s="11"/>
       <c r="G5" s="11"/>
       <c r="H5" s="11"/>
@@ -38580,23 +38580,23 @@
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" s="11"/>
-      <c r="B9" s="190" t="s">
+      <c r="B9" s="210" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="193" t="s">
+      <c r="C9" s="213" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="194"/>
-      <c r="E9" s="199" t="s">
+      <c r="D9" s="214"/>
+      <c r="E9" s="200" t="s">
         <v>23</v>
       </c>
-      <c r="F9" s="200"/>
-      <c r="G9" s="200"/>
-      <c r="H9" s="200"/>
-      <c r="I9" s="200"/>
-      <c r="J9" s="200"/>
+      <c r="F9" s="203"/>
+      <c r="G9" s="203"/>
+      <c r="H9" s="203"/>
+      <c r="I9" s="203"/>
+      <c r="J9" s="203"/>
       <c r="K9" s="201"/>
-      <c r="L9" s="199" t="s">
+      <c r="L9" s="200" t="s">
         <v>24</v>
       </c>
       <c r="M9" s="201"/>
@@ -38615,9 +38615,9 @@
     </row>
     <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11"/>
-      <c r="B10" s="191"/>
-      <c r="C10" s="195"/>
-      <c r="D10" s="196"/>
+      <c r="B10" s="211"/>
+      <c r="C10" s="215"/>
+      <c r="D10" s="216"/>
       <c r="E10" s="13" t="s">
         <v>25</v>
       </c>
@@ -38660,9 +38660,9 @@
     </row>
     <row r="11" spans="1:25" ht="119.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11"/>
-      <c r="B11" s="192"/>
-      <c r="C11" s="197"/>
-      <c r="D11" s="198"/>
+      <c r="B11" s="212"/>
+      <c r="C11" s="217"/>
+      <c r="D11" s="218"/>
       <c r="E11" s="14" t="s">
         <v>34</v>
       </c>
@@ -39022,7 +39022,7 @@
       <c r="B17" s="202" t="s">
         <v>254</v>
       </c>
-      <c r="C17" s="200"/>
+      <c r="C17" s="203"/>
       <c r="D17" s="201"/>
       <c r="E17" s="16">
         <f t="shared" ref="E17:M17" si="0">IFERROR(AVERAGE(E12:E16),0)</f>
@@ -39075,10 +39075,10 @@
     </row>
     <row r="18" spans="1:25" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11"/>
-      <c r="B18" s="203" t="s">
+      <c r="B18" s="204" t="s">
         <v>255</v>
       </c>
-      <c r="C18" s="200"/>
+      <c r="C18" s="203"/>
       <c r="D18" s="201"/>
       <c r="E18" s="186">
         <f>E17*'Overall CO attainment'!I31/3</f>
@@ -39131,10 +39131,10 @@
     </row>
     <row r="19" spans="1:25" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="11"/>
-      <c r="B19" s="290" t="s">
+      <c r="B19" s="302" t="s">
         <v>213</v>
       </c>
-      <c r="C19" s="200"/>
+      <c r="C19" s="203"/>
       <c r="D19" s="201"/>
       <c r="E19" s="120">
         <f t="shared" ref="E19:M19" si="1">ROUNDUP((E18/3)*100,2)</f>
@@ -39249,12 +39249,12 @@
       <c r="G22" s="11"/>
       <c r="H22" s="11"/>
       <c r="I22" s="11"/>
-      <c r="J22" s="204" t="s">
+      <c r="J22" s="205" t="s">
         <v>47</v>
       </c>
-      <c r="K22" s="205"/>
-      <c r="L22" s="205"/>
-      <c r="M22" s="205"/>
+      <c r="K22" s="206"/>
+      <c r="L22" s="206"/>
+      <c r="M22" s="206"/>
       <c r="N22" s="11"/>
       <c r="O22" s="11"/>
       <c r="P22" s="11"/>
@@ -39278,12 +39278,12 @@
       <c r="G23" s="11"/>
       <c r="H23" s="11"/>
       <c r="I23" s="11"/>
-      <c r="J23" s="206" t="s">
+      <c r="J23" s="207" t="s">
         <v>48</v>
       </c>
-      <c r="K23" s="207"/>
-      <c r="L23" s="207"/>
-      <c r="M23" s="208"/>
+      <c r="K23" s="208"/>
+      <c r="L23" s="208"/>
+      <c r="M23" s="209"/>
       <c r="N23" s="25"/>
       <c r="O23" s="25"/>
       <c r="P23" s="11"/>

</xml_diff>